<commit_message>
Revert "Merge branch 'integration' into feature/manojkumar/vo"
This reverts commit 5ba1c025c6561df71da4eb82e2f86cb2364cf2e6, reversing
changes made to d2b47e348f66713e537749e692a6594855c3f924.
</commit_message>
<xml_diff>
--- a/resources/Youth_beta.xlsx
+++ b/resources/Youth_beta.xlsx
@@ -9,9 +9,34 @@
     <sheet name="UserData" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="YouthClubMembers" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="7">
+  <si>
+    <t>yco2606271134m2@maildrop.cc</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>yco2606271134m1@maildrop.cc</t>
+  </si>
+  <si>
+    <t>yco2606271136m4@maildrop.cc</t>
+  </si>
+  <si>
+    <t>yco2606271136m3@maildrop.cc</t>
+  </si>
+  <si>
+    <t>yco2606271140m5@maildrop.cc</t>
+  </si>
+  <si>
+    <t>yco2606271140m6@maildrop.cc</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1321,24 +1346,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="0">
         <is>
           <t>Youth Club Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="0">
         <is>
           <t>Status</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>